<commit_message>
fix(import): flexibilize invoice header mapping and add missing number column in test data
</commit_message>
<xml_diff>
--- a/test-data/invoices.xlsx
+++ b/test-data/invoices.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,15 +407,18 @@
         <v>Entidad</v>
       </c>
       <c r="C1" t="str">
+        <v>Número</v>
+      </c>
+      <c r="D1" t="str">
         <v>Tipo</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Monto</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Vencimiento</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Estado</v>
       </c>
     </row>
@@ -427,15 +430,18 @@
         <v>Cliente Alpha S.A.</v>
       </c>
       <c r="C2" t="str">
+        <v>A-0001</v>
+      </c>
+      <c r="D2" t="str">
         <v>Venta</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>350000</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>15/01/2026</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Cobrada</v>
       </c>
     </row>
@@ -447,15 +453,18 @@
         <v>Cliente Beta Corp</v>
       </c>
       <c r="C3" t="str">
+        <v>A-0002</v>
+      </c>
+      <c r="D3" t="str">
         <v>Venta</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>450000</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>25/01/2026</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Cobrada</v>
       </c>
     </row>
@@ -467,15 +476,18 @@
         <v>Inmobiliaria Local</v>
       </c>
       <c r="C4" t="str">
+        <v>B-5521</v>
+      </c>
+      <c r="D4" t="str">
         <v>Compra</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>100000</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>10/01/2026</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Pagada</v>
       </c>
     </row>
@@ -487,15 +499,18 @@
         <v>Tech Solutions</v>
       </c>
       <c r="C5" t="str">
+        <v>A-1200</v>
+      </c>
+      <c r="D5" t="str">
         <v>Venta</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>120000</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>20/02/2026</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Pendiente</v>
       </c>
     </row>
@@ -507,15 +522,18 @@
         <v>Tech Solutions</v>
       </c>
       <c r="C6" t="str">
+        <v>C-0091</v>
+      </c>
+      <c r="D6" t="str">
         <v>Compra</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>15000</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>22/01/2026</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>Pagada</v>
       </c>
     </row>
@@ -527,15 +545,18 @@
         <v>Cliente Alpha S.A.</v>
       </c>
       <c r="C7" t="str">
+        <v>A-0003</v>
+      </c>
+      <c r="D7" t="str">
         <v>Venta</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>350000</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>15/02/2026</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Cobrada</v>
       </c>
     </row>
@@ -547,15 +568,18 @@
         <v>Cliente Beta Corp</v>
       </c>
       <c r="C8" t="str">
+        <v>A-0004</v>
+      </c>
+      <c r="D8" t="str">
         <v>Venta</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>450000</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>25/02/2026</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Cobrada</v>
       </c>
     </row>
@@ -567,15 +591,18 @@
         <v>Inmobiliaria Local</v>
       </c>
       <c r="C9" t="str">
+        <v>B-5522</v>
+      </c>
+      <c r="D9" t="str">
         <v>Compra</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>120000</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>10/02/2026</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Pagada</v>
       </c>
     </row>
@@ -587,15 +614,18 @@
         <v>Cliente Gamma (CRÍTICO)</v>
       </c>
       <c r="C10" t="str">
+        <v>A-9901</v>
+      </c>
+      <c r="D10" t="str">
         <v>Venta</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>900000</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>05/03/2026</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>Pendiente</v>
       </c>
     </row>
@@ -607,21 +637,24 @@
         <v>Proveedor Importación</v>
       </c>
       <c r="C11" t="str">
+        <v>IMP-550</v>
+      </c>
+      <c r="D11" t="str">
         <v>Compra</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>1500000</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>15/03/2026</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Pendiente</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(import): align excel import with manual entry flow and handle contado payments
</commit_message>
<xml_diff>
--- a/test-data/invoices.xlsx
+++ b/test-data/invoices.xlsx
@@ -419,7 +419,7 @@
         <v>Vencimiento</v>
       </c>
       <c r="G1" t="str">
-        <v>Estado</v>
+        <v>Condición</v>
       </c>
     </row>
     <row r="2">
@@ -442,7 +442,7 @@
         <v>15/01/2026</v>
       </c>
       <c r="G2" t="str">
-        <v>Cobrada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="3">
@@ -465,7 +465,7 @@
         <v>25/01/2026</v>
       </c>
       <c r="G3" t="str">
-        <v>Cobrada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         <v>10/01/2026</v>
       </c>
       <c r="G4" t="str">
-        <v>Pagada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="5">
@@ -511,7 +511,7 @@
         <v>20/02/2026</v>
       </c>
       <c r="G5" t="str">
-        <v>Pendiente</v>
+        <v>Cuenta Corriente</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         <v>22/01/2026</v>
       </c>
       <c r="G6" t="str">
-        <v>Pagada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="7">
@@ -557,7 +557,7 @@
         <v>15/02/2026</v>
       </c>
       <c r="G7" t="str">
-        <v>Cobrada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="8">
@@ -580,7 +580,7 @@
         <v>25/02/2026</v>
       </c>
       <c r="G8" t="str">
-        <v>Cobrada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="9">
@@ -603,7 +603,7 @@
         <v>10/02/2026</v>
       </c>
       <c r="G9" t="str">
-        <v>Pagada</v>
+        <v>Contado</v>
       </c>
     </row>
     <row r="10">
@@ -626,7 +626,7 @@
         <v>05/03/2026</v>
       </c>
       <c r="G10" t="str">
-        <v>Pendiente</v>
+        <v>Cuenta Corriente</v>
       </c>
     </row>
     <row r="11">
@@ -649,7 +649,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="G11" t="str">
-        <v>Pendiente</v>
+        <v>Cuenta Corriente</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(import): support explicit document types (Factura, NC, ND) in excel import
</commit_message>
<xml_diff>
--- a/test-data/invoices.xlsx
+++ b/test-data/invoices.xlsx
@@ -397,264 +397,297 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Tipo Documento</v>
+      </c>
+      <c r="B1" t="str">
         <v>Fecha</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Entidad</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Número</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Tipo</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Monto</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Vencimiento</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Condición</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B2" t="str">
         <v>01/01/2026</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Cliente Alpha S.A.</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>A-0001</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Venta</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>350000</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>15/01/2026</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B3" t="str">
         <v>10/01/2026</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>Cliente Beta Corp</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>A-0002</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Venta</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>450000</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>25/01/2026</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B4" t="str">
         <v>10/01/2026</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>Inmobiliaria Local</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>B-5521</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Compra</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>100000</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>10/01/2026</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Nota de Crédito</v>
+      </c>
+      <c r="B5" t="str">
         <v>20/01/2026</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>Tech Solutions</v>
       </c>
-      <c r="C5" t="str">
-        <v>A-1200</v>
-      </c>
       <c r="D5" t="str">
+        <v>NC-001</v>
+      </c>
+      <c r="E5" t="str">
         <v>Venta</v>
       </c>
-      <c r="E5">
-        <v>120000</v>
-      </c>
-      <c r="F5" t="str">
-        <v>20/02/2026</v>
+      <c r="F5">
+        <v>50000</v>
       </c>
       <c r="G5" t="str">
+        <v>20/01/2026</v>
+      </c>
+      <c r="H5" t="str">
         <v>Cuenta Corriente</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Nota de Débito</v>
+      </c>
+      <c r="B6" t="str">
         <v>22/01/2026</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>Tech Solutions</v>
       </c>
-      <c r="C6" t="str">
-        <v>C-0091</v>
-      </c>
       <c r="D6" t="str">
+        <v>ND-044</v>
+      </c>
+      <c r="E6" t="str">
         <v>Compra</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>15000</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>22/01/2026</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B7" t="str">
         <v>01/02/2026</v>
       </c>
-      <c r="B7" t="str">
+      <c r="C7" t="str">
         <v>Cliente Alpha S.A.</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>A-0003</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Venta</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>350000</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>15/02/2026</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Nota de Crédito</v>
+      </c>
+      <c r="B8" t="str">
         <v>10/02/2026</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>Cliente Beta Corp</v>
       </c>
-      <c r="C8" t="str">
-        <v>A-0004</v>
-      </c>
       <c r="D8" t="str">
+        <v>NC-002</v>
+      </c>
+      <c r="E8" t="str">
         <v>Venta</v>
       </c>
-      <c r="E8">
-        <v>450000</v>
-      </c>
-      <c r="F8" t="str">
-        <v>25/02/2026</v>
+      <c r="F8">
+        <v>25000</v>
       </c>
       <c r="G8" t="str">
+        <v>10/02/2026</v>
+      </c>
+      <c r="H8" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B9" t="str">
         <v>10/02/2026</v>
       </c>
-      <c r="B9" t="str">
+      <c r="C9" t="str">
         <v>Inmobiliaria Local</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>B-5522</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Compra</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>120000</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>10/02/2026</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>Contado</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B10" t="str">
         <v>01/03/2026</v>
       </c>
-      <c r="B10" t="str">
+      <c r="C10" t="str">
         <v>Cliente Gamma (CRÍTICO)</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>A-9901</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Venta</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>900000</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>05/03/2026</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>Cuenta Corriente</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Factura</v>
+      </c>
+      <c r="B11" t="str">
         <v>10/03/2026</v>
       </c>
-      <c r="B11" t="str">
+      <c r="C11" t="str">
         <v>Proveedor Importación</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>IMP-550</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Compra</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>1500000</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>15/03/2026</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>Cuenta Corriente</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>